<commit_message>
New readme and some other doc and testing work
</commit_message>
<xml_diff>
--- a/change_plans.xlsx
+++ b/change_plans.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mepdw\Git\BristolFE-v2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mepdw\Git\BristolFE-v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39A9EACC-4159-48B1-8527-ABE906A1B52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCD4C99F-7446-4C51-A524-72FD89D60178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4ED4B7BA-7B1F-440F-83D9-1CC24D319783}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4ED4B7BA-7B1F-440F-83D9-1CC24D319783}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="104">
   <si>
     <t>fn_ABAQUS.m</t>
   </si>
@@ -257,9 +257,6 @@
     <t>Should make it so that general 3d bdry can be specified rather than just a cuboid (to provide same functionality as 2d versions)</t>
   </si>
   <si>
-    <t>Generalise to 3D as well, based on facet surface</t>
-  </si>
-  <si>
     <t>Tidy up. Remove options to call obsolete versions</t>
   </si>
   <si>
@@ -293,9 +290,6 @@
     <t>Finish it! But in general, should be in code/internal functions.</t>
   </si>
   <si>
-    <t>code/code/internal/abaqus</t>
-  </si>
-  <si>
     <t>Need generalising for 3D - used in subdomain stuff</t>
   </si>
   <si>
@@ -326,12 +320,6 @@
     <t>Put all non-essential functions into code\internal if not required for general use</t>
   </si>
   <si>
-    <t>Todo</t>
-  </si>
-  <si>
-    <t>Generalise 2D one. Shouldn't be hard as key functions for getting distance to surface already done</t>
-  </si>
-  <si>
     <t>fn_3d_create_smooth_random_blob.m</t>
   </si>
   <si>
@@ -339,13 +327,34 @@
   </si>
   <si>
     <t>fn_2d_random_walk</t>
+  </si>
+  <si>
+    <t>code/internal/abaqus</t>
+  </si>
+  <si>
+    <t>Generalise 2D one, based on facet surface description</t>
+  </si>
+  <si>
+    <t>Needs facet surface description, then use internal function for getting distance to surface</t>
+  </si>
+  <si>
+    <t>Part done</t>
+  </si>
+  <si>
+    <t>Done - minor issue re-subdomains</t>
+  </si>
+  <si>
+    <t>Should work for 2d and 3d but latter needs checking</t>
+  </si>
+  <si>
+    <t>Done - needs checking in 3d</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -360,12 +369,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Consolas"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -388,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -397,9 +400,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -445,14 +445,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9F00509C-FE5D-4C03-9CC3-9ADEE36D4BF5}" name="Table1" displayName="Table1" ref="A10:F62" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
-  <autoFilter ref="A10:F62" xr:uid="{9F00509C-FE5D-4C03-9CC3-9ADEE36D4BF5}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="code"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9F00509C-FE5D-4C03-9CC3-9ADEE36D4BF5}" name="Table1" displayName="Table1" ref="A10:F61" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+  <autoFilter ref="A10:F61" xr:uid="{9F00509C-FE5D-4C03-9CC3-9ADEE36D4BF5}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A11:F61">
     <sortCondition ref="A10:A61"/>
   </sortState>
@@ -785,44 +779,44 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E84AA5C-B324-48B5-AC26-CDBD29B21C26}">
-  <dimension ref="A1:F62"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F61"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="43.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="19" style="1" customWidth="1"/>
-    <col min="6" max="6" width="78.7109375" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="8.7109375" style="1"/>
+    <col min="1" max="1" width="43.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.1796875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="44.26953125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="78.7265625" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>56</v>
       </c>
@@ -842,9 +836,9 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>44</v>
@@ -853,60 +847,57 @@
         <v>37</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>37</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>45</v>
+        <v>101</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>37</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>89</v>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>96</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>44</v>
@@ -915,29 +906,26 @@
         <v>37</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>37</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>44</v>
@@ -946,353 +934,383 @@
         <v>37</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>38</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>2</v>
+        <v>89</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>3</v>
+        <v>94</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>52</v>
+        <v>100</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>38</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" s="1" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="30" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>81</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
+      <c r="E36" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D38" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>81</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
-        <v>17</v>
+        <v>58</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E40" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>44</v>
@@ -1301,98 +1319,104 @@
         <v>40</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A49" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A50" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E50" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F43" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>44</v>
@@ -1401,109 +1425,79 @@
         <v>40</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="F53" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D54" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="E54" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>81</v>
+        <v>28</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>31</v>
       </c>
@@ -1514,13 +1508,13 @@
         <v>37</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>32</v>
       </c>
@@ -1531,13 +1525,13 @@
         <v>37</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F59" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>33</v>
       </c>
@@ -1548,13 +1542,13 @@
         <v>40</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>34</v>
       </c>
@@ -1565,21 +1559,7 @@
         <v>40</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>